<commit_message>
Progress updated images added
</commit_message>
<xml_diff>
--- a/01_Mechanical_Design/MectoSYS_Proto_BOM_Rev5.xlsx
+++ b/01_Mechanical_Design/MectoSYS_Proto_BOM_Rev5.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/920e4c882022e26f/Personal Folder/00_Startup/00_MectoSYS_Repo/01_Mechanical_Design/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="8_{0B3F33A1-8F31-4523-A43E-34761EEA0610}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3250D3E7-C534-41D7-9D1D-10246D0A29C0}"/>
+  <xr:revisionPtr revIDLastSave="26" documentId="8_{0B3F33A1-8F31-4523-A43E-34761EEA0610}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3DB898DF-1415-4A10-AC34-4F83258503C2}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{DED39E1D-C519-45F6-B07F-353D55FF40C1}"/>
   </bookViews>
@@ -18,10 +18,19 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">BOM!$B$1:$B$92</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -134,7 +143,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="960" uniqueCount="368">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="980" uniqueCount="368">
   <si>
     <t>Sr No</t>
   </si>
@@ -1708,7 +1717,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="73">
+  <cellXfs count="67">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1790,45 +1799,6 @@
     <xf numFmtId="0" fontId="11" fillId="5" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1869,17 +1839,40 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -2618,90 +2611,90 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:49">
-      <c r="A1" s="41" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="41" t="s">
+      <c r="A1" s="58" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="58" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="41" t="s">
+      <c r="C1" s="58" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="43" t="s">
+      <c r="D1" s="60" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="41" t="s">
+      <c r="E1" s="58" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="48" t="s">
+      <c r="F1" s="65" t="s">
         <v>356</v>
       </c>
-      <c r="G1" s="44" t="s">
+      <c r="G1" s="61" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="45" t="s">
+      <c r="H1" s="62" t="s">
         <v>340</v>
       </c>
-      <c r="I1" s="46"/>
-      <c r="J1" s="46"/>
-      <c r="K1" s="46"/>
-      <c r="L1" s="46"/>
-      <c r="M1" s="46"/>
-      <c r="N1" s="46"/>
-      <c r="O1" s="47"/>
+      <c r="I1" s="63"/>
+      <c r="J1" s="63"/>
+      <c r="K1" s="63"/>
+      <c r="L1" s="63"/>
+      <c r="M1" s="63"/>
+      <c r="N1" s="63"/>
+      <c r="O1" s="64"/>
       <c r="P1" s="31"/>
-      <c r="Q1" s="45" t="s">
+      <c r="Q1" s="62" t="s">
         <v>341</v>
       </c>
-      <c r="R1" s="46"/>
-      <c r="S1" s="46"/>
-      <c r="T1" s="46"/>
-      <c r="U1" s="46"/>
-      <c r="V1" s="46"/>
-      <c r="W1" s="46"/>
-      <c r="X1" s="47"/>
+      <c r="R1" s="63"/>
+      <c r="S1" s="63"/>
+      <c r="T1" s="63"/>
+      <c r="U1" s="63"/>
+      <c r="V1" s="63"/>
+      <c r="W1" s="63"/>
+      <c r="X1" s="64"/>
       <c r="Y1" s="31"/>
-      <c r="Z1" s="45" t="s">
+      <c r="Z1" s="62" t="s">
         <v>342</v>
       </c>
-      <c r="AA1" s="46"/>
-      <c r="AB1" s="46"/>
-      <c r="AC1" s="46"/>
-      <c r="AD1" s="46"/>
-      <c r="AE1" s="46"/>
-      <c r="AF1" s="46"/>
-      <c r="AG1" s="47"/>
+      <c r="AA1" s="63"/>
+      <c r="AB1" s="63"/>
+      <c r="AC1" s="63"/>
+      <c r="AD1" s="63"/>
+      <c r="AE1" s="63"/>
+      <c r="AF1" s="63"/>
+      <c r="AG1" s="64"/>
       <c r="AH1" s="31"/>
-      <c r="AI1" s="45" t="s">
+      <c r="AI1" s="62" t="s">
         <v>343</v>
       </c>
-      <c r="AJ1" s="46"/>
-      <c r="AK1" s="46"/>
-      <c r="AL1" s="46"/>
-      <c r="AM1" s="46"/>
-      <c r="AN1" s="46"/>
-      <c r="AO1" s="46"/>
-      <c r="AP1" s="47"/>
+      <c r="AJ1" s="63"/>
+      <c r="AK1" s="63"/>
+      <c r="AL1" s="63"/>
+      <c r="AM1" s="63"/>
+      <c r="AN1" s="63"/>
+      <c r="AO1" s="63"/>
+      <c r="AP1" s="64"/>
       <c r="AQ1" s="25"/>
-      <c r="AR1" s="41" t="s">
+      <c r="AR1" s="58" t="s">
         <v>13</v>
       </c>
-      <c r="AS1" s="41" t="s">
+      <c r="AS1" s="58" t="s">
         <v>14</v>
       </c>
-      <c r="AT1" s="41"/>
-      <c r="AU1" s="41"/>
-      <c r="AV1" s="41"/>
-      <c r="AW1" s="41"/>
+      <c r="AT1" s="58"/>
+      <c r="AU1" s="58"/>
+      <c r="AV1" s="58"/>
+      <c r="AW1" s="58"/>
     </row>
     <row r="2" spans="1:49">
-      <c r="A2" s="41"/>
-      <c r="B2" s="41"/>
-      <c r="C2" s="41"/>
-      <c r="D2" s="43"/>
-      <c r="E2" s="41"/>
-      <c r="F2" s="49"/>
-      <c r="G2" s="44"/>
+      <c r="A2" s="58"/>
+      <c r="B2" s="58"/>
+      <c r="C2" s="58"/>
+      <c r="D2" s="60"/>
+      <c r="E2" s="58"/>
+      <c r="F2" s="66"/>
+      <c r="G2" s="61"/>
       <c r="H2" s="26" t="s">
         <v>6</v>
       </c>
@@ -2802,12 +2795,12 @@
         <v>12</v>
       </c>
       <c r="AQ2" s="25"/>
-      <c r="AR2" s="41"/>
-      <c r="AS2" s="41"/>
-      <c r="AT2" s="41"/>
-      <c r="AU2" s="41"/>
-      <c r="AV2" s="41"/>
-      <c r="AW2" s="41"/>
+      <c r="AR2" s="58"/>
+      <c r="AS2" s="58"/>
+      <c r="AT2" s="58"/>
+      <c r="AU2" s="58"/>
+      <c r="AV2" s="58"/>
+      <c r="AW2" s="58"/>
     </row>
     <row r="3" spans="1:49">
       <c r="A3" s="4">
@@ -4013,7 +4006,9 @@
       <c r="E13" s="21" t="s">
         <v>240</v>
       </c>
-      <c r="F13" s="35"/>
+      <c r="F13" s="35" t="s">
+        <v>357</v>
+      </c>
       <c r="G13" s="24"/>
       <c r="H13" s="28" t="s">
         <v>227</v>
@@ -4121,7 +4116,9 @@
       <c r="E14" s="21" t="s">
         <v>240</v>
       </c>
-      <c r="F14" s="35"/>
+      <c r="F14" s="35" t="s">
+        <v>357</v>
+      </c>
       <c r="G14" s="24"/>
       <c r="H14" s="28" t="s">
         <v>227</v>
@@ -4229,7 +4226,9 @@
       <c r="E15" s="21" t="s">
         <v>231</v>
       </c>
-      <c r="F15" s="35"/>
+      <c r="F15" s="35" t="s">
+        <v>357</v>
+      </c>
       <c r="G15" s="24"/>
       <c r="H15" s="28" t="s">
         <v>227</v>
@@ -4328,7 +4327,7 @@
       </c>
       <c r="E16" s="21"/>
       <c r="F16" s="35"/>
-      <c r="G16" s="42" t="s">
+      <c r="G16" s="59" t="s">
         <v>354</v>
       </c>
       <c r="H16" s="28" t="s">
@@ -4414,7 +4413,7 @@
       </c>
       <c r="E17" s="21"/>
       <c r="F17" s="35"/>
-      <c r="G17" s="42"/>
+      <c r="G17" s="59"/>
       <c r="H17" s="28" t="s">
         <v>344</v>
       </c>
@@ -4504,7 +4503,7 @@
       </c>
       <c r="E18" s="21"/>
       <c r="F18" s="35"/>
-      <c r="G18" s="42"/>
+      <c r="G18" s="59"/>
       <c r="H18" s="28" t="s">
         <v>344</v>
       </c>
@@ -4592,7 +4591,7 @@
       </c>
       <c r="E19" s="21"/>
       <c r="F19" s="35"/>
-      <c r="G19" s="42"/>
+      <c r="G19" s="59"/>
       <c r="H19" s="28" t="s">
         <v>344</v>
       </c>
@@ -4684,7 +4683,7 @@
       </c>
       <c r="E20" s="21"/>
       <c r="F20" s="35"/>
-      <c r="G20" s="42"/>
+      <c r="G20" s="59"/>
       <c r="H20" s="28" t="s">
         <v>344</v>
       </c>
@@ -4774,7 +4773,7 @@
       </c>
       <c r="E21" s="21"/>
       <c r="F21" s="35"/>
-      <c r="G21" s="42"/>
+      <c r="G21" s="59"/>
       <c r="H21" s="28" t="s">
         <v>344</v>
       </c>
@@ -4858,7 +4857,7 @@
       </c>
       <c r="E22" s="21"/>
       <c r="F22" s="35"/>
-      <c r="G22" s="42"/>
+      <c r="G22" s="59"/>
       <c r="H22" s="28" t="s">
         <v>344</v>
       </c>
@@ -4948,7 +4947,7 @@
       </c>
       <c r="E23" s="21"/>
       <c r="F23" s="35"/>
-      <c r="G23" s="42"/>
+      <c r="G23" s="59"/>
       <c r="H23" s="28" t="s">
         <v>344</v>
       </c>
@@ -5034,7 +5033,7 @@
       </c>
       <c r="E24" s="21"/>
       <c r="F24" s="35"/>
-      <c r="G24" s="42"/>
+      <c r="G24" s="59"/>
       <c r="H24" s="28" t="s">
         <v>344</v>
       </c>
@@ -5120,7 +5119,7 @@
       </c>
       <c r="E25" s="21"/>
       <c r="F25" s="35"/>
-      <c r="G25" s="42"/>
+      <c r="G25" s="59"/>
       <c r="H25" s="28" t="s">
         <v>344</v>
       </c>
@@ -5208,7 +5207,7 @@
       </c>
       <c r="E26" s="21"/>
       <c r="F26" s="35"/>
-      <c r="G26" s="42"/>
+      <c r="G26" s="59"/>
       <c r="H26" s="28" t="s">
         <v>344</v>
       </c>
@@ -5298,7 +5297,7 @@
       </c>
       <c r="E27" s="21"/>
       <c r="F27" s="35"/>
-      <c r="G27" s="42"/>
+      <c r="G27" s="59"/>
       <c r="H27" s="28" t="s">
         <v>344</v>
       </c>
@@ -5390,7 +5389,7 @@
       </c>
       <c r="E28" s="21"/>
       <c r="F28" s="35"/>
-      <c r="G28" s="42"/>
+      <c r="G28" s="59"/>
       <c r="H28" s="28" t="s">
         <v>344</v>
       </c>
@@ -5480,7 +5479,7 @@
       </c>
       <c r="E29" s="21"/>
       <c r="F29" s="35"/>
-      <c r="G29" s="42"/>
+      <c r="G29" s="59"/>
       <c r="H29" s="28" t="s">
         <v>344</v>
       </c>
@@ -6628,7 +6627,7 @@
       </c>
       <c r="E40" s="21"/>
       <c r="F40" s="35"/>
-      <c r="G40" s="42" t="s">
+      <c r="G40" s="59" t="s">
         <v>354</v>
       </c>
       <c r="H40" s="28" t="s">
@@ -6710,7 +6709,7 @@
       </c>
       <c r="E41" s="21"/>
       <c r="F41" s="35"/>
-      <c r="G41" s="42"/>
+      <c r="G41" s="59"/>
       <c r="H41" s="28" t="s">
         <v>344</v>
       </c>
@@ -6790,7 +6789,7 @@
       </c>
       <c r="E42" s="21"/>
       <c r="F42" s="35"/>
-      <c r="G42" s="42"/>
+      <c r="G42" s="59"/>
       <c r="H42" s="28" t="s">
         <v>344</v>
       </c>
@@ -6872,7 +6871,7 @@
       </c>
       <c r="E43" s="21"/>
       <c r="F43" s="35"/>
-      <c r="G43" s="42"/>
+      <c r="G43" s="59"/>
       <c r="H43" s="28" t="s">
         <v>344</v>
       </c>
@@ -6952,7 +6951,7 @@
       </c>
       <c r="E44" s="21"/>
       <c r="F44" s="35"/>
-      <c r="G44" s="42"/>
+      <c r="G44" s="59"/>
       <c r="H44" s="28" t="s">
         <v>344</v>
       </c>
@@ -7032,7 +7031,7 @@
       </c>
       <c r="E45" s="21"/>
       <c r="F45" s="35"/>
-      <c r="G45" s="42"/>
+      <c r="G45" s="59"/>
       <c r="H45" s="28" t="s">
         <v>344</v>
       </c>
@@ -7112,7 +7111,7 @@
       </c>
       <c r="E46" s="21"/>
       <c r="F46" s="35"/>
-      <c r="G46" s="42"/>
+      <c r="G46" s="59"/>
       <c r="H46" s="28" t="s">
         <v>344</v>
       </c>
@@ -7192,7 +7191,7 @@
       </c>
       <c r="E47" s="21"/>
       <c r="F47" s="35"/>
-      <c r="G47" s="42"/>
+      <c r="G47" s="59"/>
       <c r="H47" s="28" t="s">
         <v>344</v>
       </c>
@@ -7270,7 +7269,7 @@
       </c>
       <c r="E48" s="21"/>
       <c r="F48" s="35"/>
-      <c r="G48" s="42"/>
+      <c r="G48" s="59"/>
       <c r="H48" s="28" t="s">
         <v>344</v>
       </c>
@@ -7350,7 +7349,7 @@
       </c>
       <c r="E49" s="21"/>
       <c r="F49" s="35"/>
-      <c r="G49" s="42"/>
+      <c r="G49" s="59"/>
       <c r="H49" s="28" t="s">
         <v>344</v>
       </c>
@@ -7428,7 +7427,7 @@
       </c>
       <c r="E50" s="21"/>
       <c r="F50" s="35"/>
-      <c r="G50" s="42"/>
+      <c r="G50" s="59"/>
       <c r="H50" s="28" t="s">
         <v>344</v>
       </c>
@@ -7506,7 +7505,7 @@
       </c>
       <c r="E51" s="21"/>
       <c r="F51" s="35"/>
-      <c r="G51" s="42"/>
+      <c r="G51" s="59"/>
       <c r="H51" s="28" t="s">
         <v>344</v>
       </c>
@@ -7584,7 +7583,7 @@
       </c>
       <c r="E52" s="21"/>
       <c r="F52" s="35"/>
-      <c r="G52" s="42"/>
+      <c r="G52" s="59"/>
       <c r="H52" s="28" t="s">
         <v>344</v>
       </c>
@@ -7662,7 +7661,7 @@
       </c>
       <c r="E53" s="21"/>
       <c r="F53" s="35"/>
-      <c r="G53" s="42"/>
+      <c r="G53" s="59"/>
       <c r="H53" s="28" t="s">
         <v>344</v>
       </c>
@@ -7740,7 +7739,7 @@
       </c>
       <c r="E54" s="21"/>
       <c r="F54" s="35"/>
-      <c r="G54" s="42"/>
+      <c r="G54" s="59"/>
       <c r="H54" s="28" t="s">
         <v>344</v>
       </c>
@@ -7818,7 +7817,7 @@
       </c>
       <c r="E55" s="21"/>
       <c r="F55" s="35"/>
-      <c r="G55" s="42"/>
+      <c r="G55" s="59"/>
       <c r="H55" s="28" t="s">
         <v>344</v>
       </c>
@@ -7896,7 +7895,7 @@
       </c>
       <c r="E56" s="21"/>
       <c r="F56" s="35"/>
-      <c r="G56" s="42"/>
+      <c r="G56" s="59"/>
       <c r="H56" s="28" t="s">
         <v>344</v>
       </c>
@@ -7972,7 +7971,7 @@
       </c>
       <c r="E57" s="21"/>
       <c r="F57" s="35"/>
-      <c r="G57" s="42"/>
+      <c r="G57" s="59"/>
       <c r="H57" s="28" t="s">
         <v>344</v>
       </c>
@@ -8869,7 +8868,9 @@
         <v>268</v>
       </c>
       <c r="E66" s="21"/>
-      <c r="F66" s="35"/>
+      <c r="F66" s="35" t="s">
+        <v>357</v>
+      </c>
       <c r="G66" s="24" t="s">
         <v>355</v>
       </c>
@@ -8953,7 +8954,9 @@
         <v>271</v>
       </c>
       <c r="E67" s="21"/>
-      <c r="F67" s="35"/>
+      <c r="F67" s="35" t="s">
+        <v>357</v>
+      </c>
       <c r="G67" s="24"/>
       <c r="H67" s="28" t="s">
         <v>349</v>
@@ -9055,7 +9058,9 @@
         <v>274</v>
       </c>
       <c r="E68" s="21"/>
-      <c r="F68" s="35"/>
+      <c r="F68" s="35" t="s">
+        <v>357</v>
+      </c>
       <c r="G68" s="24"/>
       <c r="H68" s="28" t="s">
         <v>349</v>
@@ -9264,7 +9269,9 @@
         <v>280</v>
       </c>
       <c r="E70" s="21"/>
-      <c r="F70" s="35"/>
+      <c r="F70" s="35" t="s">
+        <v>357</v>
+      </c>
       <c r="G70" s="24"/>
       <c r="H70" s="28" t="s">
         <v>349</v>
@@ -9366,7 +9373,9 @@
         <v>283</v>
       </c>
       <c r="E71" s="21"/>
-      <c r="F71" s="35"/>
+      <c r="F71" s="35" t="s">
+        <v>357</v>
+      </c>
       <c r="G71" s="24"/>
       <c r="H71" s="28" t="s">
         <v>349</v>
@@ -9473,7 +9482,9 @@
         <v>286</v>
       </c>
       <c r="E72" s="21"/>
-      <c r="F72" s="35"/>
+      <c r="F72" s="35" t="s">
+        <v>357</v>
+      </c>
       <c r="G72" s="24"/>
       <c r="H72" s="28" t="s">
         <v>349</v>
@@ -9575,8 +9586,8 @@
         <v>289</v>
       </c>
       <c r="E73" s="21"/>
-      <c r="F73" s="37"/>
-      <c r="G73" s="39" t="s">
+      <c r="F73" s="35"/>
+      <c r="G73" s="56" t="s">
         <v>355</v>
       </c>
       <c r="H73" s="28" t="s">
@@ -9659,8 +9670,10 @@
         <v>291</v>
       </c>
       <c r="E74" s="21"/>
-      <c r="F74" s="38"/>
-      <c r="G74" s="40"/>
+      <c r="F74" s="35" t="s">
+        <v>357</v>
+      </c>
+      <c r="G74" s="57"/>
       <c r="H74" s="28" t="s">
         <v>349</v>
       </c>
@@ -9743,7 +9756,9 @@
       <c r="E75" s="21" t="s">
         <v>231</v>
       </c>
-      <c r="F75" s="35"/>
+      <c r="F75" s="35" t="s">
+        <v>357</v>
+      </c>
       <c r="G75" s="24"/>
       <c r="H75" s="28" t="s">
         <v>349</v>
@@ -9852,7 +9867,9 @@
         <v>298</v>
       </c>
       <c r="E76" s="21"/>
-      <c r="F76" s="35"/>
+      <c r="F76" s="35" t="s">
+        <v>357</v>
+      </c>
       <c r="G76" s="24"/>
       <c r="H76" s="28" t="s">
         <v>349</v>
@@ -9954,7 +9971,9 @@
         <v>300</v>
       </c>
       <c r="E77" s="21"/>
-      <c r="F77" s="35"/>
+      <c r="F77" s="35" t="s">
+        <v>357</v>
+      </c>
       <c r="G77" s="24"/>
       <c r="H77" s="28" t="s">
         <v>349</v>
@@ -10531,7 +10550,9 @@
         <v>312</v>
       </c>
       <c r="E83" s="21"/>
-      <c r="F83" s="35"/>
+      <c r="F83" s="35" t="s">
+        <v>357</v>
+      </c>
       <c r="G83" s="24"/>
       <c r="H83" s="30" t="s">
         <v>95</v>
@@ -10742,7 +10763,9 @@
         <v>332</v>
       </c>
       <c r="E85" s="21"/>
-      <c r="F85" s="35"/>
+      <c r="F85" s="35" t="s">
+        <v>357</v>
+      </c>
       <c r="G85" s="24"/>
       <c r="H85" s="28" t="s">
         <v>333</v>
@@ -10844,7 +10867,9 @@
         <v>336</v>
       </c>
       <c r="E86" s="21"/>
-      <c r="F86" s="35"/>
+      <c r="F86" s="35" t="s">
+        <v>357</v>
+      </c>
       <c r="G86" s="24"/>
       <c r="H86" s="28" t="s">
         <v>333</v>
@@ -11143,7 +11168,9 @@
         <v>217</v>
       </c>
       <c r="E89" s="21"/>
-      <c r="F89" s="35"/>
+      <c r="F89" s="35" t="s">
+        <v>357</v>
+      </c>
       <c r="G89" s="24"/>
       <c r="H89" s="30" t="s">
         <v>203</v>
@@ -11243,7 +11270,9 @@
         <v>194</v>
       </c>
       <c r="E90" s="21"/>
-      <c r="F90" s="35"/>
+      <c r="F90" s="35" t="s">
+        <v>357</v>
+      </c>
       <c r="G90" s="24"/>
       <c r="H90" s="30" t="s">
         <v>203</v>
@@ -11343,7 +11372,9 @@
         <v>202</v>
       </c>
       <c r="E91" s="21"/>
-      <c r="F91" s="35"/>
+      <c r="F91" s="35" t="s">
+        <v>357</v>
+      </c>
       <c r="G91" s="24"/>
       <c r="H91" s="30" t="s">
         <v>203</v>
@@ -11430,111 +11461,113 @@
       <c r="AW91" s="3"/>
     </row>
     <row r="92" spans="1:49">
-      <c r="A92" s="50">
+      <c r="A92" s="37">
         <v>90</v>
       </c>
-      <c r="B92" s="51" t="s">
+      <c r="B92" s="38" t="s">
         <v>206</v>
       </c>
-      <c r="C92" s="52"/>
-      <c r="D92" s="52" t="s">
+      <c r="C92" s="39"/>
+      <c r="D92" s="39" t="s">
         <v>207</v>
       </c>
-      <c r="E92" s="53"/>
-      <c r="F92" s="37"/>
-      <c r="G92" s="54"/>
-      <c r="H92" s="55" t="s">
+      <c r="E92" s="40"/>
+      <c r="F92" s="35" t="s">
+        <v>357</v>
+      </c>
+      <c r="G92" s="41"/>
+      <c r="H92" s="42" t="s">
         <v>203</v>
       </c>
-      <c r="I92" s="56" t="s">
+      <c r="I92" s="43" t="s">
         <v>94</v>
       </c>
-      <c r="J92" s="57" t="s">
-        <v>8</v>
-      </c>
-      <c r="K92" s="58"/>
-      <c r="L92" s="58">
+      <c r="J92" s="44" t="s">
+        <v>8</v>
+      </c>
+      <c r="K92" s="45"/>
+      <c r="L92" s="45">
         <v>9.09</v>
       </c>
-      <c r="M92" s="58">
+      <c r="M92" s="45">
         <v>1</v>
       </c>
-      <c r="N92" s="58"/>
-      <c r="O92" s="59">
+      <c r="N92" s="45"/>
+      <c r="O92" s="46">
         <f t="shared" si="11"/>
         <v>9.09</v>
       </c>
-      <c r="P92" s="60"/>
-      <c r="Q92" s="61" t="s">
+      <c r="P92" s="47"/>
+      <c r="Q92" s="48" t="s">
         <v>93</v>
       </c>
-      <c r="R92" s="62">
+      <c r="R92" s="49">
         <v>1</v>
       </c>
-      <c r="S92" s="63" t="s">
-        <v>8</v>
-      </c>
-      <c r="T92" s="52"/>
-      <c r="U92" s="52">
+      <c r="S92" s="50" t="s">
+        <v>8</v>
+      </c>
+      <c r="T92" s="39"/>
+      <c r="U92" s="39">
         <v>12.7</v>
       </c>
-      <c r="V92" s="52">
+      <c r="V92" s="39">
         <v>1</v>
       </c>
-      <c r="W92" s="52">
-        <v>0</v>
-      </c>
-      <c r="X92" s="64">
+      <c r="W92" s="39">
+        <v>0</v>
+      </c>
+      <c r="X92" s="51">
         <f t="shared" si="7"/>
         <v>12.7</v>
       </c>
-      <c r="Y92" s="60"/>
-      <c r="Z92" s="55" t="s">
+      <c r="Y92" s="47"/>
+      <c r="Z92" s="42" t="s">
         <v>95</v>
       </c>
-      <c r="AA92" s="65" t="s">
+      <c r="AA92" s="52" t="s">
         <v>94</v>
       </c>
-      <c r="AB92" s="57" t="s">
-        <v>8</v>
-      </c>
-      <c r="AC92" s="58"/>
-      <c r="AD92" s="58">
+      <c r="AB92" s="44" t="s">
+        <v>8</v>
+      </c>
+      <c r="AC92" s="45"/>
+      <c r="AD92" s="45">
         <v>12.7</v>
       </c>
-      <c r="AE92" s="58">
+      <c r="AE92" s="45">
         <v>1</v>
       </c>
-      <c r="AF92" s="58"/>
-      <c r="AG92" s="64">
+      <c r="AF92" s="45"/>
+      <c r="AG92" s="51">
         <f t="shared" si="8"/>
         <v>12.7</v>
       </c>
-      <c r="AH92" s="60"/>
-      <c r="AI92" s="55"/>
-      <c r="AJ92" s="65"/>
-      <c r="AK92" s="57"/>
-      <c r="AL92" s="58"/>
-      <c r="AM92" s="58"/>
-      <c r="AN92" s="58"/>
-      <c r="AO92" s="58"/>
-      <c r="AP92" s="66"/>
-      <c r="AQ92" s="67"/>
-      <c r="AR92" s="58"/>
-      <c r="AS92" s="58"/>
-      <c r="AT92" s="58"/>
-      <c r="AU92" s="58"/>
-      <c r="AV92" s="58"/>
-      <c r="AW92" s="58"/>
+      <c r="AH92" s="47"/>
+      <c r="AI92" s="42"/>
+      <c r="AJ92" s="52"/>
+      <c r="AK92" s="44"/>
+      <c r="AL92" s="45"/>
+      <c r="AM92" s="45"/>
+      <c r="AN92" s="45"/>
+      <c r="AO92" s="45"/>
+      <c r="AP92" s="53"/>
+      <c r="AQ92" s="54"/>
+      <c r="AR92" s="45"/>
+      <c r="AS92" s="45"/>
+      <c r="AT92" s="45"/>
+      <c r="AU92" s="45"/>
+      <c r="AV92" s="45"/>
+      <c r="AW92" s="45"/>
     </row>
     <row r="93" spans="1:49">
-      <c r="A93" s="68">
+      <c r="A93" s="4">
         <v>91</v>
       </c>
-      <c r="B93" s="69" t="s">
+      <c r="B93" s="6" t="s">
         <v>360</v>
       </c>
-      <c r="C93" s="69" t="s">
+      <c r="C93" s="6" t="s">
         <v>361</v>
       </c>
       <c r="D93" s="17">
@@ -11543,20 +11576,20 @@
       <c r="E93" s="3"/>
       <c r="F93" s="3"/>
       <c r="G93" s="3"/>
-      <c r="H93" s="70" t="s">
+      <c r="H93" s="17" t="s">
         <v>362</v>
       </c>
       <c r="I93" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="J93" s="71" t="s">
+      <c r="J93" s="55" t="s">
         <v>8</v>
       </c>
       <c r="K93" s="3"/>
-      <c r="L93" s="72">
+      <c r="L93" s="3">
         <v>47.72</v>
       </c>
-      <c r="M93" s="72">
+      <c r="M93" s="3">
         <v>2</v>
       </c>
       <c r="N93" s="3"/>
@@ -11600,13 +11633,13 @@
       <c r="AW93" s="3"/>
     </row>
     <row r="94" spans="1:49">
-      <c r="A94" s="68">
+      <c r="A94" s="4">
         <v>92</v>
       </c>
-      <c r="B94" s="69" t="s">
+      <c r="B94" s="6" t="s">
         <v>363</v>
       </c>
-      <c r="C94" s="69" t="s">
+      <c r="C94" s="6" t="s">
         <v>229</v>
       </c>
       <c r="D94" s="3" t="s">
@@ -11615,20 +11648,20 @@
       <c r="E94" s="3"/>
       <c r="F94" s="3"/>
       <c r="G94" s="3"/>
-      <c r="H94" s="70" t="s">
+      <c r="H94" s="17" t="s">
         <v>211</v>
       </c>
       <c r="I94" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="J94" s="71" t="s">
+      <c r="J94" s="55" t="s">
         <v>8</v>
       </c>
       <c r="K94" s="3"/>
-      <c r="L94" s="72">
+      <c r="L94" s="3">
         <v>96.63</v>
       </c>
-      <c r="M94" s="72">
+      <c r="M94" s="3">
         <v>2</v>
       </c>
       <c r="N94" s="3"/>
@@ -11672,13 +11705,13 @@
       <c r="AW94" s="3"/>
     </row>
     <row r="95" spans="1:49">
-      <c r="A95" s="68">
+      <c r="A95" s="4">
         <v>93</v>
       </c>
-      <c r="B95" s="69" t="s">
+      <c r="B95" s="6" t="s">
         <v>365</v>
       </c>
-      <c r="C95" s="69" t="s">
+      <c r="C95" s="6" t="s">
         <v>366</v>
       </c>
       <c r="D95" s="3" t="s">
@@ -11687,20 +11720,20 @@
       <c r="E95" s="3"/>
       <c r="F95" s="3"/>
       <c r="G95" s="3"/>
-      <c r="H95" s="70" t="s">
+      <c r="H95" s="17" t="s">
         <v>211</v>
       </c>
       <c r="I95" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="J95" s="71" t="s">
+      <c r="J95" s="55" t="s">
         <v>8</v>
       </c>
       <c r="K95" s="3"/>
-      <c r="L95" s="72">
+      <c r="L95" s="3">
         <v>100.83</v>
       </c>
-      <c r="M95" s="72">
+      <c r="M95" s="3">
         <v>1</v>
       </c>
       <c r="N95" s="3"/>

</xml_diff>